<commit_message>
Add stg_performance: type all 32 performance columns with sentinel handling and profiled decimals
</commit_message>
<xml_diff>
--- a/resources/file_layout_pre_july_2026 - use this.xlsx
+++ b/resources/file_layout_pre_july_2026 - use this.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2b9f5a77d560c584/Documents/Courses/Building a product governance portfolio/Resourses/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2b9f5a77d560c584/Documents/Courses/mortgage-portfolio-governance/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{D7C3A213-42EC-48A8-9061-6E8FDA558764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{962705AE-2FE0-48BD-A672-623FB964A437}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Origination Data File" sheetId="1" r:id="rId1"/>
@@ -406,6 +406,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>